<commit_message>
Drift sweep landed: all 15 register drifts closed (D11-D14 ruled as recommended)
Contradictions fixed (conservation equation aligned to produce;
spine about widened to lower-or-same layer; description status
machine-only; ownership-flip wording modernized; class overview
trimmed to one line each). Stale pointers cleared (logic contract
subsumed; IOUs marked closed; companion lines added for
KG3/KG4/Lenses/Flows; L1_* wording). Rulings landed: grain
opportunistic qualifier; referenced_keys = lens #17 never stored;
edge-direction convention ratified (references point toward
stability, containment parent->child); D1 accounting widened to
layers 2-4; L0 two-directions clarified in the flows map.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (drift sweep)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The one law ratified (Sunny): nothing in the graph is ever physically deleted
Change supersedes, current is derived, retired nodes remain valid
targets — SCD2/catalog-soft-delete/event-sourcing basis. S2 closed
(no orphans exist), S3 reduced to a retention default (forever;
pruning is a ruled act). H1 + H2 closed in the register. Layer 2's
regenerability rule amended: rebuild supersedes, never deletes.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1024,7 +1024,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: name-keyed identity + one-law supersession</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: one-law supersession retains versions; retention forever by default, pruning ruled</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CHANGE pass CLOSED: S4 correspondence + S5 staleness economics ratified; H7/H8 closed
Four holes died in one pass (H1 identity, H2 witness/retention,
H7 correspondence, H8 economics) — all descendants of one question:
what survives change. Remaining passes: EDGES (H3,H4,H5),
SAFETY (H6,H11), SCALE/OPS (H9,H10).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1216,7 +1216,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: S4 overlap-maximal correspondence, closed outcomes, human rules ambiguity</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: S5 budgeted queue, usage-weighted priority, counted backlog</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SAFETY pass CLOSED: PHI boundary, the one redaction exception to the one law, tenancy — H6/H11 closed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1184,7 +1184,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: PHI boundary (verbatim-after-redaction, both doors) + the one ruled redaction exception w/ tombstone event</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: tenancy sentence in the doc; egress = de-identified aggregates by explicit decision</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCALE/OPS pass CLOSED — all four passes done; the open register stands at 15/15 + 11/11
The hardening phase is complete: Level-1 design ratified end to
end, every seam and lifecycle contracted, every hole from the
holistic critique ruled and landed. Register remains the standing
home for future findings.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -486,6 +486,18 @@
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>A hole in this register is owned; a hole in someone's memory is a hope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>REGISTER CLOSED 2026-09-05: 15/15 drifts, 11/11 holes. New findings open new rows; this file stays the standing register for future passes.</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1292,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: envelope as registry data + lens materialization modes</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1324,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05: run outcome + per-artifact atomicity; resume = the staleness worklist</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ambiguity review landed: A1-A10 as register rows (evidence-based, each with its undecidable test case)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -10,6 +10,7 @@
     <sheet name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Drifts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Holes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ambiguities" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +55,11 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B8860B"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -79,6 +85,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1363,4 +1372,322 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Ambiguity (evidence-based)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Undecidable test case</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Readings that both comply</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>db-node ownership when two sources share a db</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>epic + org extracts both declare db CLARITY — whose extract owns the db node, whose as_of?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>first-wins | per-source duplicates | source-neutral container</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>L1 identity includes db name; db names are not stable. FAMILY: also the resolution matching rules (case folding PAT_ENC vs pat_enc; values-map key types '3' vs 3) are delegated but never stated</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>org migrates CLARITYPRDDB -&gt; CLARITY: same source, same tables</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>all identities break (mass retire+create) | identity = (source, schema, table), db as property</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>duplicate scope names within one file break the name-key</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>WITH Base in statement 1 AND statement 3 — legal SQL, one name-key</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>qualify by position (unstable) | collision counted | last-wins</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>unnamed scopes (subqueries) have no identity for attachments</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>a description about a subquery scope — nothing forbids it</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>implicitly forbidden (unstated) | positional identity (unstable)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>asked on ambiguous match: how many about edges</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>five candidates, user picks one — five touches or none or one?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>about-all (usage inflation corrupts flywheel lenses) | none-until-confirmed | only-the-chosen</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>'current is derived' — the selection algorithm is never stated</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>chain: machine, human, machine-proposed, human, machine-rejected-in-middle</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>latest-non-proposed | latest-human-or-accepted | others — same answer on easy chains, different on hard ones</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>regenerability depends on retained extracts; retention duty unassigned</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>rebuild needed in year 2; DBA's snapshot folder gone</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>AIVIA retains every snapshot (where?) | rebuild from a FRESH extract (a different graph)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>bootstrap ordering: org extract before vendor extract</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>org extract references epic tables that do not exist yet</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>refuse (mandatory intake order, unstated) | accept w/ pending targets (a dangling state the layer otherwise never has)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>produce-run conservation scope across classes</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>a run ships 40 descriptions + 3 term nominations — one equation or per-class?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>single equation (killed-lines meaningless for terms) | per-class accounting</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>'a named human confirmation' of a send — named by whom, qualified how</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>steward accepted; an engagement admin clicks send</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>any authenticated human | role-qualified | must be the accepter</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Disambiguation clause amended (models first, J2 restored) + A1-A10 ruled model-first
Every rule now a total mapping over a declared domain with its
witness example; A6's totality check yields a non-emptiness proof;
A4 resolved as a domain bound rather than a branch; A10's role
qualification declared an intent judgment per the typed exception.
All ten register ambiguity rows closed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1440,7 +1440,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>CLOSED 2026-09-05 (model-first ruling in doc)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Solo-stretch _OPEN flags filed as register rows A11-A15 (the HITL law: flagged, never decided)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1380,7 +1380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1687,6 +1687,141 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>A11 (F2-A)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>unnamed final-scope attachment: a file's final SELECT scope has no name; A4 says artifacts attach to named nodes only</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>produce describes usp_diabetic_visits' final scope — attach where?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>attach to the FILE node | mint a conventional name (::final)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — drafts use file-attachment UNRULED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>A12 (F3-A)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>scope-mediated join compliance: a practiced join to a #temp holding another table's ids</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ENCOUNTER_DX joined to #Recent (ENCOUNTER ids) — judge the underlying ENCOUNTER_DX-ENCOUNTER pair or only direct pairs?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>direct table-table pairs only | resolve through scopes</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — drafts use direct-only UNRULED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>A13 (F4-A)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>the deterministic floor's sentence grammar is not ratified — the design states WHAT facts the floor voices, not how</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>what exact sentence does the #Recent floor emit?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ratify a floor grammar (seeded by the field-proven composer) | keep expect/forbid substrings as the only contract</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — F4 asserts facts via substrings only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>A14 (F6-A)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>malformed fk group: quarantine-and-proceed (contract §6) vs whole-extract refusal (LC-F5 atomicity instinct)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>fk group with ordinals 1,3 — accept the extract?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>quarantine + proceed + counted | refuse the extract</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — F6 drafts quarantine per §6 UNRULED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>A15 (F5-A)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>per-target export column headers are unbound (rules ratified: zero custom attrs + prefix; headers = build binding)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>the exact CSV headers for catalog_a</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>bind at build from the term-propose precedent | ratify now</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — F5 asserts rules, not headers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
A11 RULED (Sunny): ::delivery naming w/ DBA list for plural emitters; A12 placed ON HOLD (projection contingent)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1710,7 +1710,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>OPEN — drafts use file-attachment UNRULED</t>
+          <t>RULED 2026-09-05 (Sunny): single emitter -&gt; file::delivery; plural -&gt; delivery_n each + DBA ruling list</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>RULED 2026-09-05: through-scope (real forensics); entailed: PROJECTION structure kind added to KG2</t>
+          <t>ON HOLD (Sunny 2026-09-05): ruled through-scope, then reopened for further discussion; PROJECTION amendment contingent</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A14 + A15 RULED (Sunny): quarantine+DBA-alert (HITL) for malformed fk groups; export headers bind at the build slice — AMBIGUITY SHEET FULLY CLOSED
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Open_Register.xlsx
+++ b/AIVIA_Design/L1_Open_Register.xlsx
@@ -1791,7 +1791,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>OPEN — F6 drafts quarantine per §6 UNRULED</t>
+          <t>RULED 2026-09-05 (Sunny): quarantine + count + DBA alert (HITL); refusals reserved for identity-level problems</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>OPEN — F5 asserts rules, not headers</t>
+          <t>RULED 2026-09-05 (Sunny): headers bind at the build slice from the term-propose precedent</t>
         </is>
       </c>
     </row>

</xml_diff>